<commit_message>
v0.15.20: derive the barcode annealing tail from the file and refuse a file that does not state it
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/04_mame_custom_barcodes.xlsx
+++ b/src-tauri/samples/mame/04_mame_custom_barcodes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="barcodes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="barcodes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AAGAAAGTTGTCGGTGTCTTTGTG</t>
+          <t>TATCTGACCTTCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TCGATTCCGTTTGTAGTCGTCTGT</t>
+          <t>GCATACGTAACCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GAGTCTTGTGTCCCAGTTACCAGG</t>
+          <t>AACTTGCATAGCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TTCGGATTCTATCGTGTTTCCCTA</t>
+          <t>TGACCTAAGGTCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CTTGTCCAGGGTTTGTGTAACCTT</t>
+          <t>CCGTATATAACCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TTCTCGCAAAGGCAGAAAGTAGTC</t>
+          <t>GTAACCTGCATCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GTGTTACCGTGGGAATGAATCCTT</t>
+          <t>AAGCTTACCATCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TTCAGGGAACAAACCAAGTTACGT</t>
+          <t>TTCCGGATCATCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AACTAGGCACAGCGAGTCTTGGTT</t>
+          <t>CCATTAGCATGCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AAGCGTTGAAACCTTTGTCCTCTC</t>
+          <t>GGTTAACCATGCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GTTTCATCTATCGGAGGGAATGGA</t>
+          <t>AATCCGTTAGCCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAGGTAGAAAGAAGCAGAATCGGA</t>
+          <t>GAACATACGGTCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ACGTAACTTGGTTTGTTCCCTGAA</t>
+          <t>CCCTATGACAGCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AAGGATTCATTCCCACGGTAACAC</t>
+          <t>GCTATAGCCTTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GACTACTTTCTGCCTTTGCGAGAA</t>
+          <t>TTGCAATCGATCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AAGGTTACACAAACCCTGGACAAG</t>
+          <t>CCAGTATCGGTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TAGGGAAACACGATAGAATCCGAA</t>
+          <t>GGTACCTAATGCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CCTGGTAACTGGGACACAAGACTC</t>
+          <t>AAGCTATCGCTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ACAGACGACTACAAACGGAATCGA</t>
+          <t>TTCCAGCTTAGCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CACAAAGACACCGACAACTTTCTT</t>
+          <t>AGAGTGCGGCTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.15.21: derive the barcode annealing tail from the file and refuse a file that does not state it
Derives the barcode annealing tail from the longest suffix every barcode on an axis shares, instead of two sequences hardcoded from the ispS raw data. Reproduces the deleted constants to the base on a legacy file. Removes the silent fixed-length fallback: a file whose tail cannot be derived stops the run and names the axis, the measured suffix, the floor it missed, and the rows at fault. Validate Inputs runs the same reader. Regenerates both bundled barcode workbooks, which shared nothing and only loaded through the fallback.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/04_mame_custom_barcodes.xlsx
+++ b/src-tauri/samples/mame/04_mame_custom_barcodes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="barcodes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="barcodes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AAGAAAGTTGTCGGTGTCTTTGTG</t>
+          <t>TATCTGACCTTCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TCGATTCCGTTTGTAGTCGTCTGT</t>
+          <t>GCATACGTAACCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GAGTCTTGTGTCCCAGTTACCAGG</t>
+          <t>AACTTGCATAGCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TTCGGATTCTATCGTGTTTCCCTA</t>
+          <t>TGACCTAAGGTCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CTTGTCCAGGGTTTGTGTAACCTT</t>
+          <t>CCGTATATAACCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TTCTCGCAAAGGCAGAAAGTAGTC</t>
+          <t>GTAACCTGCATCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GTGTTACCGTGGGAATGAATCCTT</t>
+          <t>AAGCTTACCATCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TTCAGGGAACAAACCAAGTTACGT</t>
+          <t>TTCCGGATCATCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AACTAGGCACAGCGAGTCTTGGTT</t>
+          <t>CCATTAGCATGCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AAGCGTTGAAACCTTTGTCCTCTC</t>
+          <t>GGTTAACCATGCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GTTTCATCTATCGGAGGGAATGGA</t>
+          <t>AATCCGTTAGCCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAGGTAGAAAGAAGCAGAATCGGA</t>
+          <t>GAACATACGGTCTATTCAGGGCGCGGTGG</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ACGTAACTTGGTTTGTTCCCTGAA</t>
+          <t>CCCTATGACAGCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AAGGATTCATTCCCACGGTAACAC</t>
+          <t>GCTATAGCCTTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GACTACTTTCTGCCTTTGCGAGAA</t>
+          <t>TTGCAATCGATCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AAGGTTACACAAACCCTGGACAAG</t>
+          <t>CCAGTATCGGTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TAGGGAAACACGATAGAATCCGAA</t>
+          <t>GGTACCTAATGCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CCTGGTAACTGGGACACAAGACTC</t>
+          <t>AAGCTATCGCTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ACAGACGACTACAAACGGAATCGA</t>
+          <t>TTCCAGCTTAGCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CACAAAGACACCGACAACTTTCTT</t>
+          <t>AGAGTGCGGCTCTCGTACCGGGGGTGCAC</t>
         </is>
       </c>
     </row>

</xml_diff>